<commit_message>
docs: WIP Master Material entries
</commit_message>
<xml_diff>
--- a/Warehouse_Operations_Portfolio.xlsx
+++ b/Warehouse_Operations_Portfolio.xlsx
@@ -8,26 +8,23 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Upgrade skill\1. Excel - Data Analytics\Project\Warehouse Operations Portfolio\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DA71BF0-0FE5-4128-A475-BF559BD5F03F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE09E6E4-D41B-4710-99A3-03A5AC08D986}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13140" firstSheet="12" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="01_Master_Part" sheetId="1" r:id="rId1"/>
+    <sheet name="01_Master_Material" sheetId="1" r:id="rId1"/>
     <sheet name="02_Master_Supplier" sheetId="2" r:id="rId2"/>
     <sheet name="03_Master_Location" sheetId="3" r:id="rId3"/>
     <sheet name="04_Purchase_Order" sheetId="4" r:id="rId4"/>
     <sheet name="05_Goods_Receipt" sheetId="5" r:id="rId5"/>
     <sheet name="06_Put_Away" sheetId="6" r:id="rId6"/>
-    <sheet name="07_Current_Inventory" sheetId="7" r:id="rId7"/>
-    <sheet name="08_Material_Request" sheetId="8" r:id="rId8"/>
-    <sheet name="09_Picking_List" sheetId="9" r:id="rId9"/>
-    <sheet name="10_Material_Issue" sheetId="10" r:id="rId10"/>
-    <sheet name="11_Stock_Card" sheetId="11" r:id="rId11"/>
-    <sheet name="12_Cycle_Count" sheetId="12" r:id="rId12"/>
-    <sheet name="13_Inventory_Adjustment" sheetId="13" r:id="rId13"/>
-    <sheet name="14_Dashboard" sheetId="14" r:id="rId14"/>
-    <sheet name="Report &amp; Insight Hasil AnysData" sheetId="15" r:id="rId15"/>
+    <sheet name="07_Material_Request" sheetId="8" r:id="rId7"/>
+    <sheet name="08_Picking_List" sheetId="9" r:id="rId8"/>
+    <sheet name="09_Goods_Issue" sheetId="10" r:id="rId9"/>
+    <sheet name="10_Stock_Card" sheetId="11" r:id="rId10"/>
+    <sheet name="11_Cycle_Count" sheetId="12" r:id="rId11"/>
+    <sheet name="12_Dashboard" sheetId="14" r:id="rId12"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -42,10 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="10">
-  <si>
-    <t>Menyimpan data seluruh material</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="95">
   <si>
     <t>Menyimpan data seluruh supplier</t>
   </si>
@@ -62,9 +56,6 @@
     <t>Menentukan lokasi penyimpanan</t>
   </si>
   <si>
-    <t>Menampilkan stok terkini</t>
-  </si>
-  <si>
     <t>Mencatat barang keluar</t>
   </si>
   <si>
@@ -72,13 +63,274 @@
   </si>
   <si>
     <t>Ringkasan KPI warehouse</t>
+  </si>
+  <si>
+    <t>01_MASTER_MATERIAL  |  Warehouse Operations in a Heavy Equipment Manufacturing Environment</t>
+  </si>
+  <si>
+    <t>Material Code</t>
+  </si>
+  <si>
+    <t>Material Description</t>
+  </si>
+  <si>
+    <t>Material Group</t>
+  </si>
+  <si>
+    <t>Base UoM</t>
+  </si>
+  <si>
+    <t>Purchase UoM</t>
+  </si>
+  <si>
+    <t>Conversion Factor (Purchase to Base)</t>
+  </si>
+  <si>
+    <t>Primary Supplier Code</t>
+  </si>
+  <si>
+    <t>Standard Cost (per Base UoM)</t>
+  </si>
+  <si>
+    <t>ABC Classification</t>
+  </si>
+  <si>
+    <t>Criticality Flag</t>
+  </si>
+  <si>
+    <t>Storage/Handling Class</t>
+  </si>
+  <si>
+    <t>Min Stock Level</t>
+  </si>
+  <si>
+    <t>Max Stock Level</t>
+  </si>
+  <si>
+    <t>Lead Time (Days)</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>MAT-00001</t>
+  </si>
+  <si>
+    <t>Hydraulic Cylinder Seal Kit 80mm</t>
+  </si>
+  <si>
+    <t>Hydraulic Components</t>
+  </si>
+  <si>
+    <t>PCS</t>
+  </si>
+  <si>
+    <t>BOX</t>
+  </si>
+  <si>
+    <t>SUP-0012</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>Critical Spare</t>
+  </si>
+  <si>
+    <t>Standard</t>
+  </si>
+  <si>
+    <t>Active</t>
+  </si>
+  <si>
+    <t>MAT-00002</t>
+  </si>
+  <si>
+    <t>Steel Plate 10mm x 2m x 1m</t>
+  </si>
+  <si>
+    <t>Raw Steel</t>
+  </si>
+  <si>
+    <t>SUP-0005</t>
+  </si>
+  <si>
+    <t>Heavy/Bulk</t>
+  </si>
+  <si>
+    <t>MAT-00003</t>
+  </si>
+  <si>
+    <t>Engine Oil Filter (Cat 320D)</t>
+  </si>
+  <si>
+    <t>Engine Parts</t>
+  </si>
+  <si>
+    <t>SUP-0021</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>MAT-00004</t>
+  </si>
+  <si>
+    <t>Hex Bolt M12x50 Grade 8.8</t>
+  </si>
+  <si>
+    <t>Fasteners</t>
+  </si>
+  <si>
+    <t>SUP-0009</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>MAT-00005</t>
+  </si>
+  <si>
+    <t>Industrial Degreaser 20L</t>
+  </si>
+  <si>
+    <t>Consumables</t>
+  </si>
+  <si>
+    <t>LTR</t>
+  </si>
+  <si>
+    <t>SUP-0014</t>
+  </si>
+  <si>
+    <t>Hazardous</t>
+  </si>
+  <si>
+    <t>MAT-00006</t>
+  </si>
+  <si>
+    <t>Track Roller Assembly (Komatsu D65)</t>
+  </si>
+  <si>
+    <t>MAT-00007</t>
+  </si>
+  <si>
+    <t>Air Filter Element - Primary</t>
+  </si>
+  <si>
+    <t>MAT-00008</t>
+  </si>
+  <si>
+    <t>Hydraulic Hose 1/2in x 3m</t>
+  </si>
+  <si>
+    <t>MAT-00009</t>
+  </si>
+  <si>
+    <t>Grease Cartridge NLGI2 400g</t>
+  </si>
+  <si>
+    <t>MAT-00010</t>
+  </si>
+  <si>
+    <t>Welding Electrode E7018 3.2mm</t>
+  </si>
+  <si>
+    <t>KG</t>
+  </si>
+  <si>
+    <t>MAT-00011</t>
+  </si>
+  <si>
+    <t>Final Drive Motor (Excavator PC200)</t>
+  </si>
+  <si>
+    <t>Finished Spares</t>
+  </si>
+  <si>
+    <t>SUP-0033</t>
+  </si>
+  <si>
+    <t>MAT-00012</t>
+  </si>
+  <si>
+    <t>Bucket Teeth (CAT style)</t>
+  </si>
+  <si>
+    <t>MAT-00013</t>
+  </si>
+  <si>
+    <t>Radiator Coolant 20L</t>
+  </si>
+  <si>
+    <t>MAT-00014</t>
+  </si>
+  <si>
+    <t>Flat Washer M12 Zinc Plated</t>
+  </si>
+  <si>
+    <t>MAT-00015</t>
+  </si>
+  <si>
+    <t>Turbocharger Assembly (Cat C15)</t>
+  </si>
+  <si>
+    <t>MAT-00016</t>
+  </si>
+  <si>
+    <t>V-Belt A-Section 1250mm</t>
+  </si>
+  <si>
+    <t>MAT-00017</t>
+  </si>
+  <si>
+    <t>Steel I-Beam 6m Length</t>
+  </si>
+  <si>
+    <t>MAT-00018</t>
+  </si>
+  <si>
+    <t>Cabin Air Filter</t>
+  </si>
+  <si>
+    <t>MAT-00019</t>
+  </si>
+  <si>
+    <t>Bearing 6205-2RS</t>
+  </si>
+  <si>
+    <t>MAT-00020</t>
+  </si>
+  <si>
+    <t>Undercarriage Chain Link Assembly</t>
+  </si>
+  <si>
+    <t>Inactive</t>
+  </si>
+  <si>
+    <t>Notes / Data Dictionary</t>
+  </si>
+  <si>
+    <t>- Material Code: Primary key. Format MAT-##### used consistently across all worksheets.</t>
+  </si>
+  <si>
+    <t>- ABC Classification: A = high value/usage (tight control, frequent cycle count), B = moderate, C = low value/high volume (loose control).</t>
+  </si>
+  <si>
+    <t>- Criticality Flag: 'Critical Spare' = stockout risk causes production/machine downtime; monitored more closely on Dashboard.</t>
+  </si>
+  <si>
+    <t>- Conversion Factor: Multiply Purchase UoM quantity by this factor to obtain Base UoM quantity (used in PO/GR reconciliation).</t>
+  </si>
+  <si>
+    <t>- Status: Only 'Active' materials should be used in new transactions (PO, Picking, Issue).</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -86,16 +338,58 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="9"/>
+      <color rgb="FF595959"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF2E75B6"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -103,17 +397,89 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB7B7B7"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB7B7B7"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB7B7B7"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB7B7B7"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="3" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="4" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="6">
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="thin">
+          <color rgb="FFB7B7B7"/>
+        </left>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <right style="thin">
+          <color rgb="FFB7B7B7"/>
+        </right>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FFC00000"/>
+        <name val="Arial"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFD9D9D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -124,6 +490,30 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BE6A9852-60D4-4C66-8A7A-2A7C0A2B3B6E}" name="tbl_MasterMaterial" displayName="tbl_MasterMaterial" ref="A3:O23">
+  <autoFilter ref="A3:O23" xr:uid="{BE6A9852-60D4-4C66-8A7A-2A7C0A2B3B6E}"/>
+  <tableColumns count="15">
+    <tableColumn id="1" xr3:uid="{F06BE5B9-22B9-48F2-924F-2C915E1203C7}" name="Material Code" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{A37F0F00-EA5A-48E2-B47C-E0FC342313D4}" name="Material Description" dataDxfId="0"/>
+    <tableColumn id="3" xr3:uid="{96B447C5-85FC-41F9-BD64-7BC716DCD55B}" name="Material Group" dataDxfId="1"/>
+    <tableColumn id="4" xr3:uid="{1D99F23F-22DA-4DE3-8F44-D6FA922054BA}" name="Base UoM"/>
+    <tableColumn id="5" xr3:uid="{19408CD1-C13E-4DF7-AA14-7740AD42FF9D}" name="Purchase UoM"/>
+    <tableColumn id="6" xr3:uid="{7BD5224A-B5A6-421E-A682-000CE933B858}" name="Conversion Factor (Purchase to Base)"/>
+    <tableColumn id="7" xr3:uid="{1879E6A1-BA80-4BDC-8AC5-607DDEC12936}" name="Primary Supplier Code"/>
+    <tableColumn id="8" xr3:uid="{2BBC43DA-B41F-43FA-B2CC-54A781579160}" name="Standard Cost (per Base UoM)"/>
+    <tableColumn id="9" xr3:uid="{0694E72F-5791-4767-B302-9410B16F972D}" name="ABC Classification"/>
+    <tableColumn id="10" xr3:uid="{19845E0C-E010-406D-B570-B1465124B111}" name="Criticality Flag"/>
+    <tableColumn id="11" xr3:uid="{A42A9606-BE97-41FC-8D78-7A371C795B31}" name="Storage/Handling Class"/>
+    <tableColumn id="12" xr3:uid="{EF94269D-2F67-4C4C-9516-299B8E297B6A}" name="Min Stock Level"/>
+    <tableColumn id="13" xr3:uid="{CA2A04A3-F8A3-4B8E-ACB0-8ACEDE15D8F9}" name="Max Stock Level"/>
+    <tableColumn id="14" xr3:uid="{D89767DE-A26F-4EE6-9673-091B7F887BB2}" name="Lead Time (Days)"/>
+    <tableColumn id="15" xr3:uid="{027F9326-927F-4874-B9CD-B903907AFD45}" name="Status"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -390,36 +780,1110 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1"/>
+  <dimension ref="A1:O31"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="15.28515625" customWidth="1"/>
+    <col min="2" max="2" width="34.85546875" customWidth="1"/>
+    <col min="3" max="3" width="20" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.42578125" customWidth="1"/>
+    <col min="5" max="5" width="11.28515625" customWidth="1"/>
+    <col min="6" max="6" width="21.140625" customWidth="1"/>
+    <col min="7" max="7" width="16.85546875" customWidth="1"/>
+    <col min="8" max="8" width="15.140625" customWidth="1"/>
+    <col min="9" max="9" width="13.140625" customWidth="1"/>
+    <col min="10" max="10" width="16" customWidth="1"/>
+    <col min="11" max="11" width="17.28515625" customWidth="1"/>
+    <col min="12" max="12" width="12.5703125" customWidth="1"/>
+    <col min="13" max="13" width="10.42578125" customWidth="1"/>
+    <col min="14" max="14" width="11.5703125" customWidth="1"/>
+    <col min="15" max="15" width="10.5703125" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>0</v>
+    <row r="1" spans="1:15" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+      <c r="K1" s="2"/>
+      <c r="L1" s="2"/>
+      <c r="M1" s="2"/>
+      <c r="N1" s="2"/>
+      <c r="O1" s="2"/>
+    </row>
+    <row r="3" spans="1:15" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="L3" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="M3" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="N3" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="O3" s="3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A4" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="F4" s="5">
+        <v>10</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="H4" s="6">
+        <v>145.5</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="K4" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="L4" s="5">
+        <v>20</v>
+      </c>
+      <c r="M4" s="5">
+        <v>100</v>
+      </c>
+      <c r="N4" s="5">
+        <v>14</v>
+      </c>
+      <c r="O4" s="4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" s="5">
+        <v>1</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="H5" s="6">
+        <v>320</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="J5" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="K5" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="L5" s="5">
+        <v>10</v>
+      </c>
+      <c r="M5" s="5">
+        <v>50</v>
+      </c>
+      <c r="N5" s="5">
+        <v>21</v>
+      </c>
+      <c r="O5" s="4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="F6" s="5">
+        <v>24</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="H6" s="6">
+        <v>18.75</v>
+      </c>
+      <c r="I6" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="J6" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="K6" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="L6" s="5">
+        <v>50</v>
+      </c>
+      <c r="M6" s="5">
+        <v>300</v>
+      </c>
+      <c r="N6" s="5">
+        <v>7</v>
+      </c>
+      <c r="O6" s="4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="F7" s="5">
+        <v>100</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="H7" s="6">
+        <v>0.35</v>
+      </c>
+      <c r="I7" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="J7" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="K7" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="L7" s="5">
+        <v>500</v>
+      </c>
+      <c r="M7" s="5">
+        <v>5000</v>
+      </c>
+      <c r="N7" s="5">
+        <v>10</v>
+      </c>
+      <c r="O7" s="4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="F8" s="5">
+        <v>20</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="H8" s="6">
+        <v>4.2</v>
+      </c>
+      <c r="I8" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="J8" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="K8" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="L8" s="5">
+        <v>40</v>
+      </c>
+      <c r="M8" s="5">
+        <v>200</v>
+      </c>
+      <c r="N8" s="5">
+        <v>5</v>
+      </c>
+      <c r="O8" s="4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="F9" s="5">
+        <v>1</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="H9" s="6">
+        <v>890</v>
+      </c>
+      <c r="I9" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="J9" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="K9" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="L9" s="5">
+        <v>4</v>
+      </c>
+      <c r="M9" s="5">
+        <v>20</v>
+      </c>
+      <c r="N9" s="5">
+        <v>30</v>
+      </c>
+      <c r="O9" s="4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="F10" s="5">
+        <v>12</v>
+      </c>
+      <c r="G10" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="H10" s="6">
+        <v>32.1</v>
+      </c>
+      <c r="I10" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="J10" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="K10" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="L10" s="5">
+        <v>30</v>
+      </c>
+      <c r="M10" s="5">
+        <v>150</v>
+      </c>
+      <c r="N10" s="5">
+        <v>10</v>
+      </c>
+      <c r="O10" s="4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A11" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="F11" s="5">
+        <v>1</v>
+      </c>
+      <c r="G11" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="H11" s="6">
+        <v>54.9</v>
+      </c>
+      <c r="I11" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="J11" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="K11" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="L11" s="5">
+        <v>15</v>
+      </c>
+      <c r="M11" s="5">
+        <v>80</v>
+      </c>
+      <c r="N11" s="5">
+        <v>12</v>
+      </c>
+      <c r="O11" s="4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A12" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="F12" s="5">
+        <v>12</v>
+      </c>
+      <c r="G12" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="H12" s="6">
+        <v>6.8</v>
+      </c>
+      <c r="I12" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="J12" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="K12" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="L12" s="5">
+        <v>60</v>
+      </c>
+      <c r="M12" s="5">
+        <v>400</v>
+      </c>
+      <c r="N12" s="5">
+        <v>5</v>
+      </c>
+      <c r="O12" s="4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A13" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="F13" s="5">
+        <v>5</v>
+      </c>
+      <c r="G13" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="H13" s="6">
+        <v>3.95</v>
+      </c>
+      <c r="I13" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="J13" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="K13" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="L13" s="5">
+        <v>100</v>
+      </c>
+      <c r="M13" s="5">
+        <v>600</v>
+      </c>
+      <c r="N13" s="5">
+        <v>7</v>
+      </c>
+      <c r="O13" s="4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A14" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="F14" s="5">
+        <v>1</v>
+      </c>
+      <c r="G14" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="H14" s="6">
+        <v>2450</v>
+      </c>
+      <c r="I14" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="J14" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="K14" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="L14" s="5">
+        <v>2</v>
+      </c>
+      <c r="M14" s="5">
+        <v>10</v>
+      </c>
+      <c r="N14" s="5">
+        <v>45</v>
+      </c>
+      <c r="O14" s="4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A15" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="F15" s="5">
+        <v>10</v>
+      </c>
+      <c r="G15" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="H15" s="6">
+        <v>42</v>
+      </c>
+      <c r="I15" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="J15" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="K15" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="L15" s="5">
+        <v>25</v>
+      </c>
+      <c r="M15" s="5">
+        <v>120</v>
+      </c>
+      <c r="N15" s="5">
+        <v>20</v>
+      </c>
+      <c r="O15" s="4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A16" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="F16" s="5">
+        <v>20</v>
+      </c>
+      <c r="G16" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="H16" s="6">
+        <v>3.1</v>
+      </c>
+      <c r="I16" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="J16" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="K16" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="L16" s="5">
+        <v>30</v>
+      </c>
+      <c r="M16" s="5">
+        <v>150</v>
+      </c>
+      <c r="N16" s="5">
+        <v>5</v>
+      </c>
+      <c r="O16" s="4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A17" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E17" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="F17" s="5">
+        <v>200</v>
+      </c>
+      <c r="G17" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="H17" s="6">
+        <v>0.05</v>
+      </c>
+      <c r="I17" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="J17" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="K17" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="L17" s="5">
+        <v>1000</v>
+      </c>
+      <c r="M17" s="5">
+        <v>8000</v>
+      </c>
+      <c r="N17" s="5">
+        <v>10</v>
+      </c>
+      <c r="O17" s="4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A18" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E18" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="F18" s="5">
+        <v>1</v>
+      </c>
+      <c r="G18" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="H18" s="6">
+        <v>1380</v>
+      </c>
+      <c r="I18" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="J18" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="K18" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="L18" s="5">
+        <v>3</v>
+      </c>
+      <c r="M18" s="5">
+        <v>15</v>
+      </c>
+      <c r="N18" s="5">
+        <v>35</v>
+      </c>
+      <c r="O18" s="4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A19" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E19" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="F19" s="5">
+        <v>6</v>
+      </c>
+      <c r="G19" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="H19" s="6">
+        <v>12.4</v>
+      </c>
+      <c r="I19" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="J19" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="K19" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="L19" s="5">
+        <v>40</v>
+      </c>
+      <c r="M19" s="5">
+        <v>200</v>
+      </c>
+      <c r="N19" s="5">
+        <v>8</v>
+      </c>
+      <c r="O19" s="4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A20" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="F20" s="5">
+        <v>1</v>
+      </c>
+      <c r="G20" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="H20" s="6">
+        <v>610</v>
+      </c>
+      <c r="I20" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="J20" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="K20" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="L20" s="5">
+        <v>5</v>
+      </c>
+      <c r="M20" s="5">
+        <v>25</v>
+      </c>
+      <c r="N20" s="5">
+        <v>25</v>
+      </c>
+      <c r="O20" s="4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A21" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E21" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="F21" s="5">
+        <v>10</v>
+      </c>
+      <c r="G21" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="H21" s="6">
+        <v>9.6</v>
+      </c>
+      <c r="I21" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="J21" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="K21" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="L21" s="5">
+        <v>35</v>
+      </c>
+      <c r="M21" s="5">
+        <v>180</v>
+      </c>
+      <c r="N21" s="5">
+        <v>7</v>
+      </c>
+      <c r="O21" s="4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A22" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E22" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="F22" s="5">
+        <v>20</v>
+      </c>
+      <c r="G22" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="H22" s="6">
+        <v>4.75</v>
+      </c>
+      <c r="I22" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="J22" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="K22" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="L22" s="5">
+        <v>80</v>
+      </c>
+      <c r="M22" s="5">
+        <v>400</v>
+      </c>
+      <c r="N22" s="5">
+        <v>9</v>
+      </c>
+      <c r="O22" s="4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A23" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E23" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="F23" s="5">
+        <v>1</v>
+      </c>
+      <c r="G23" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="H23" s="6">
+        <v>1120</v>
+      </c>
+      <c r="I23" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="J23" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="K23" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="L23" s="5">
+        <v>2</v>
+      </c>
+      <c r="M23" s="5">
+        <v>8</v>
+      </c>
+      <c r="N23" s="5">
+        <v>40</v>
+      </c>
+      <c r="O23" s="4" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A26" s="7" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A27" s="8" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="28" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A28" s="8" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="29" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A29" s="8" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="30" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A30" s="8" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="31" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A31" s="8" t="s">
+        <v>94</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:O1"/>
+  </mergeCells>
+  <conditionalFormatting sqref="A4:O31">
+    <cfRule type="expression" dxfId="5" priority="1">
+      <formula>$O4="Inactive"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="4" priority="2">
+      <formula>$J4="Critical Spare"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I4:I31">
+    <cfRule type="expression" dxfId="3" priority="3">
+      <formula>$I4="A"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="7">
+    <dataValidation type="list" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid entry" error="Please select a value from the list." promptTitle="Status" prompt="Select material status." sqref="O4:O31" xr:uid="{A45DF13D-CE9F-46AD-88BE-5E2F01BA55D7}">
+      <formula1>"Active,Inactive"</formula1>
+    </dataValidation>
+    <dataValidation type="list" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid entry" error="Please select a value from the list." promptTitle="Storage/Handling Class" prompt="Select storage handling requirement." sqref="K4:K31" xr:uid="{E8C86EDD-4743-4074-885E-F0C2E9C9C8D7}">
+      <formula1>"Standard,Heavy/Bulk,Hazardous,Fragile"</formula1>
+    </dataValidation>
+    <dataValidation type="list" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid entry" error="Please select a value from the list." promptTitle="Criticality Flag" prompt="Flag machine-down-risk items." sqref="J4:J31" xr:uid="{12A3B5C2-8020-4216-9875-01FED103E187}">
+      <formula1>"Critical Spare,Standard"</formula1>
+    </dataValidation>
+    <dataValidation type="list" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid entry" error="Please select a value from the list." promptTitle="ABC Classification" prompt="Select ABC class (value/usage tier)." sqref="I4:I31" xr:uid="{E450422A-A08D-4FAA-AF80-FFA4B4ACD3DC}">
+      <formula1>"A,B,C"</formula1>
+    </dataValidation>
+    <dataValidation type="list" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid entry" error="Please select a value from the list." promptTitle="Purchase UoM" prompt="Select the purchase unit of measure." sqref="E4:E31" xr:uid="{7B16F677-6623-414B-B36E-DD35A8607DAF}">
+      <formula1>"PCS,KG,MTR,LTR,BOX"</formula1>
+    </dataValidation>
+    <dataValidation type="list" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid entry" error="Please select a value from the list." promptTitle="Base UoM" prompt="Select the base unit of measure." sqref="D4:D31" xr:uid="{868743FE-4C29-4F6D-8BFD-52E5CD1D616B}">
+      <formula1>"PCS,KG,MTR,LTR,BOX"</formula1>
+    </dataValidation>
+    <dataValidation type="list" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid entry" error="Please select a value from the list." promptTitle="Material Group" prompt="Select the material category." sqref="C4:C31" xr:uid="{E358F029-D9F8-4092-8610-2B511F6D7F50}">
+      <formula1>"Raw Steel,Hydraulic Components,Engine Parts,Fasteners,Consumables,Finished Spares"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE3E4AE1-8F11-41CA-9024-A0C7DC9AA7F1}">
-  <sheetPr codeName="Sheet10"/>
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C66EC62C-F615-4B55-877A-2E00EE88CF02}">
   <sheetPr codeName="Sheet11"/>
   <dimension ref="A1:A4"/>
@@ -427,12 +1891,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -440,7 +1904,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CDEE296F-75F2-4A13-9897-F22202B2F9C4}">
   <sheetPr codeName="Sheet12"/>
   <dimension ref="A1"/>
@@ -450,17 +1914,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D469330B-19AF-4D1B-8AA2-FF2FBA521645}">
-  <sheetPr codeName="Sheet13"/>
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{52F20A0A-0836-469C-B6C7-4D93916D4BDF}">
   <sheetPr codeName="Sheet14"/>
   <dimension ref="A1"/>
@@ -468,20 +1922,10 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{92BCB775-49C5-4B22-BBF9-9EE295E938AA}">
-  <sheetPr codeName="Sheet15"/>
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -494,7 +1938,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -510,7 +1954,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -526,7 +1970,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -542,7 +1986,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -558,7 +2002,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -567,22 +2011,6 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB0EDA5F-DAF7-457F-94A4-C70DA0340552}">
-  <sheetPr codeName="Sheet7"/>
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5EEA7261-B106-4D58-9AAF-59D573EFBA81}">
   <sheetPr codeName="Sheet8"/>
   <dimension ref="A1"/>
@@ -592,7 +2020,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B2F654E-B58E-40E5-8E98-D8EE3C22DE77}">
   <sheetPr codeName="Sheet9"/>
   <dimension ref="A1"/>
@@ -600,4 +2028,20 @@
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE3E4AE1-8F11-41CA-9024-A0C7DC9AA7F1}">
+  <sheetPr codeName="Sheet10"/>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>